<commit_message>
feat: Importation fichier; adaptation des fichiers template xls avec ajout de feuille de classe, matricule élève + prof etc; ajout auto de salle et alerte mode de MAJ remplacement
</commit_message>
<xml_diff>
--- a/templates/schedule.xlsx
+++ b/templates/schedule.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="EDT" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,10 +418,16 @@
       <c r="F1" t="str">
         <v>Salle</v>
       </c>
+      <c r="G1" t="str">
+        <v>Bâtiment salle</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Capacité salle</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ibrahim Diallo</v>
+        <v>Jean Traore</v>
       </c>
       <c r="B2" t="str">
         <v>3ème A</v>
@@ -433,15 +439,21 @@
         <v>Lundi</v>
       </c>
       <c r="E2" t="str">
-        <v>7h30 - 9h00</v>
+        <v>07h30 - 09h00</v>
       </c>
       <c r="F2" t="str">
         <v>Salle A1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Bloc A</v>
+      </c>
+      <c r="H2" t="str">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>